<commit_message>
New and improved results added
</commit_message>
<xml_diff>
--- a/evaluations/classification/classification_results_ensamble_test.xlsx
+++ b/evaluations/classification/classification_results_ensamble_test.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -791,7 +791,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E6" t="b">
@@ -828,16 +828,16 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>12.24</v>
+        <v>11.29</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.06560000000000001</v>
+        <v>0.0484</v>
       </c>
       <c r="R6" t="n">
-        <v>0.0919</v>
+        <v>0.073</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0727</v>
+        <v>0.0535</v>
       </c>
     </row>
     <row r="7">
@@ -854,7 +854,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>keynet_hardnet</t>
+          <t>lightglue</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -891,16 +891,16 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>9.4</v>
+        <v>5.06</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0312</v>
+        <v>0.023</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0861</v>
+        <v>0.0722</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0342</v>
+        <v>0.0283</v>
       </c>
     </row>
     <row r="8">
@@ -917,7 +917,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>ensamble</t>
         </is>
       </c>
       <c r="E8" t="b">
@@ -954,33 +954,33 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>11.29</v>
+        <v>12.24</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0484</v>
+        <v>0.06560000000000001</v>
       </c>
       <c r="R8" t="n">
-        <v>0.073</v>
+        <v>0.0919</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0535</v>
+        <v>0.0727</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CowDataset</t>
+          <t>BelugaID</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1019</v>
+        <v>6909</v>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>747</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -1017,16 +1017,16 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>2.72</v>
+        <v>9.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.9648</v>
+        <v>0.0312</v>
       </c>
       <c r="R9" t="n">
-        <v>0.9837</v>
+        <v>0.0861</v>
       </c>
       <c r="S9" t="n">
-        <v>0.969</v>
+        <v>0.0342</v>
       </c>
     </row>
     <row r="10">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>lightglue</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -1080,33 +1080,33 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>2.76</v>
+        <v>2.72</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9648</v>
       </c>
       <c r="R10" t="n">
-        <v>0.9675</v>
+        <v>0.9837</v>
       </c>
       <c r="S10" t="n">
-        <v>0.9347</v>
+        <v>0.969</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Giraffes</t>
+          <t>CowDataset</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>906</v>
+        <v>1019</v>
       </c>
       <c r="C11" t="n">
-        <v>170</v>
+        <v>12</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -1137,35 +1137,35 @@
         <v>0.5</v>
       </c>
       <c r="N11" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="O11" t="b">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>2.93</v>
+        <v>97.42</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2214</v>
+        <v>0.7104</v>
       </c>
       <c r="R11" t="n">
-        <v>0.2265</v>
+        <v>0.9044</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1995</v>
+        <v>0.7411</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Giraffes</t>
+          <t>CowDataset</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>906</v>
+        <v>1019</v>
       </c>
       <c r="C12" t="n">
-        <v>170</v>
+        <v>12</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1206,33 +1206,33 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>1.52</v>
+        <v>2.76</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.5115</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="R12" t="n">
-        <v>0.5547</v>
+        <v>0.9675</v>
       </c>
       <c r="S12" t="n">
-        <v>0.502</v>
+        <v>0.9347</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Giraffes</t>
+          <t>CowDataset</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>906</v>
+        <v>1019</v>
       </c>
       <c r="C13" t="n">
-        <v>170</v>
+        <v>12</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E13" t="b">
@@ -1269,16 +1269,16 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>4.27</v>
+        <v>91.23999999999999</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.4427</v>
+        <v>0.765</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4504</v>
+        <v>0.9044</v>
       </c>
       <c r="S13" t="n">
-        <v>0.4267</v>
+        <v>0.7894</v>
       </c>
     </row>
     <row r="14">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>keynet_hardnet</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1332,33 +1332,33 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>1.29</v>
+        <v>2.93</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.1756</v>
+        <v>0.2214</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3028</v>
+        <v>0.2265</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1542</v>
+        <v>0.1995</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>Giraffes</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2497</v>
+        <v>906</v>
       </c>
       <c r="C15" t="n">
-        <v>247</v>
+        <v>170</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>lightglue</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1395,33 +1395,33 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>5.46</v>
+        <v>1.52</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.6029</v>
+        <v>0.5115</v>
       </c>
       <c r="R15" t="n">
-        <v>0.708</v>
+        <v>0.5547</v>
       </c>
       <c r="S15" t="n">
-        <v>0.5762</v>
+        <v>0.502</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>Giraffes</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2497</v>
+        <v>906</v>
       </c>
       <c r="C16" t="n">
-        <v>247</v>
+        <v>170</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>lightglue</t>
+          <t>ensamble</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1458,33 +1458,33 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>2.15</v>
+        <v>4.27</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.5273</v>
+        <v>0.4427</v>
       </c>
       <c r="R16" t="n">
-        <v>0.6492</v>
+        <v>0.4504</v>
       </c>
       <c r="S16" t="n">
-        <v>0.4987</v>
+        <v>0.4267</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>Giraffes</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2497</v>
+        <v>906</v>
       </c>
       <c r="C17" t="n">
-        <v>247</v>
+        <v>170</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -1521,33 +1521,33 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>3.36</v>
+        <v>1.29</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.5125999999999999</v>
+        <v>0.1756</v>
       </c>
       <c r="R17" t="n">
-        <v>0.6008</v>
+        <v>0.3028</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4871</v>
+        <v>0.1542</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5499</v>
+        <v>2497</v>
       </c>
       <c r="C18" t="n">
-        <v>48</v>
+        <v>247</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>keynet_hardnet</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -1584,33 +1584,33 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>4.17</v>
+        <v>3.36</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.7467</v>
+        <v>0.5125999999999999</v>
       </c>
       <c r="R18" t="n">
-        <v>0.8673</v>
+        <v>0.6008</v>
       </c>
       <c r="S18" t="n">
-        <v>0.7459</v>
+        <v>0.4871</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5499</v>
+        <v>2497</v>
       </c>
       <c r="C19" t="n">
-        <v>48</v>
+        <v>247</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>ensamble</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1647,33 +1647,33 @@
         <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>8.369999999999999</v>
+        <v>5.46</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.7599</v>
+        <v>0.6029</v>
       </c>
       <c r="R19" t="n">
-        <v>0.8571</v>
+        <v>0.708</v>
       </c>
       <c r="S19" t="n">
-        <v>0.7574</v>
+        <v>0.5762</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5499</v>
+        <v>2497</v>
       </c>
       <c r="C20" t="n">
-        <v>48</v>
+        <v>247</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>lightglue</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1710,33 +1710,33 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>12.06</v>
+        <v>2.15</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.8146</v>
+        <v>0.5273</v>
       </c>
       <c r="R20" t="n">
-        <v>0.9108000000000001</v>
+        <v>0.6492</v>
       </c>
       <c r="S20" t="n">
-        <v>0.8128</v>
+        <v>0.4987</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NyalaData</t>
+          <t>IPanda50</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1498</v>
+        <v>5499</v>
       </c>
       <c r="C21" t="n">
-        <v>227</v>
+        <v>48</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -1773,33 +1773,33 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>4.36</v>
+        <v>4.17</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.1561</v>
+        <v>0.7467</v>
       </c>
       <c r="R21" t="n">
-        <v>0.3468</v>
+        <v>0.8673</v>
       </c>
       <c r="S21" t="n">
-        <v>0.1352</v>
+        <v>0.7459</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NyalaData</t>
+          <t>IPanda50</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1498</v>
+        <v>5499</v>
       </c>
       <c r="C22" t="n">
-        <v>227</v>
+        <v>48</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>keynet_hardnet</t>
+          <t>ensamble</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1836,33 +1836,33 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>1.63</v>
+        <v>12.06</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1387</v>
+        <v>0.8146</v>
       </c>
       <c r="R22" t="n">
-        <v>0.2977</v>
+        <v>0.9108000000000001</v>
       </c>
       <c r="S22" t="n">
-        <v>0.1167</v>
+        <v>0.8128</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NyalaData</t>
+          <t>IPanda50</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1498</v>
+        <v>5499</v>
       </c>
       <c r="C23" t="n">
-        <v>227</v>
+        <v>48</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>lightglue</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1899,16 +1899,16 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>1.88</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.1069</v>
+        <v>0.7599</v>
       </c>
       <c r="R23" t="n">
-        <v>0.2283</v>
+        <v>0.8571</v>
       </c>
       <c r="S23" t="n">
-        <v>0.0823</v>
+        <v>0.7574</v>
       </c>
     </row>
     <row r="24">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>keynet_hardnet</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1962,29 +1962,29 @@
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>2.5</v>
+        <v>1.63</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.1445</v>
+        <v>0.1387</v>
       </c>
       <c r="R24" t="n">
-        <v>0.3092</v>
+        <v>0.2977</v>
       </c>
       <c r="S24" t="n">
-        <v>0.1217</v>
+        <v>0.1167</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1668</v>
+        <v>1498</v>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>227</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2025,29 +2025,29 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>1.11</v>
+        <v>1.88</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.6977</v>
+        <v>0.1069</v>
       </c>
       <c r="R25" t="n">
-        <v>0.7806999999999999</v>
+        <v>0.2283</v>
       </c>
       <c r="S25" t="n">
-        <v>0.673</v>
+        <v>0.0823</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1668</v>
+        <v>1498</v>
       </c>
       <c r="C26" t="n">
-        <v>55</v>
+        <v>227</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2088,33 +2088,33 @@
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>2.19</v>
+        <v>2.5</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.7176</v>
+        <v>0.1445</v>
       </c>
       <c r="R26" t="n">
-        <v>0.7874</v>
+        <v>0.3092</v>
       </c>
       <c r="S26" t="n">
-        <v>0.6935</v>
+        <v>0.1217</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>655</v>
+        <v>1498</v>
       </c>
       <c r="C27" t="n">
-        <v>43</v>
+        <v>227</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>disk</t>
+          <t>ensamble</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -2151,33 +2151,33 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>0.87</v>
+        <v>4.36</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.9826</v>
+        <v>0.1561</v>
       </c>
       <c r="R27" t="n">
-        <v>0.9913</v>
+        <v>0.3468</v>
       </c>
       <c r="S27" t="n">
-        <v>0.9791</v>
+        <v>0.1352</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>SealID</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>655</v>
+        <v>1668</v>
       </c>
       <c r="C28" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>lightglue</t>
         </is>
       </c>
       <c r="E28" t="b">
@@ -2214,33 +2214,33 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>1.16</v>
+        <v>1.11</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.9913</v>
+        <v>0.6977</v>
       </c>
       <c r="R28" t="n">
-        <v>1</v>
+        <v>0.7806999999999999</v>
       </c>
       <c r="S28" t="n">
-        <v>0.9878</v>
+        <v>0.673</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>SealID</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>655</v>
+        <v>1668</v>
       </c>
       <c r="C29" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>lightglue</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E29" t="b">
@@ -2277,16 +2277,16 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>0.9</v>
+        <v>2.19</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.9043</v>
+        <v>0.7176</v>
       </c>
       <c r="R29" t="n">
-        <v>0.9565</v>
+        <v>0.7874</v>
       </c>
       <c r="S29" t="n">
-        <v>0.8963</v>
+        <v>0.6935</v>
       </c>
     </row>
     <row r="30">
@@ -2350,6 +2350,195 @@
       </c>
       <c r="S30" t="n">
         <v>0.9162</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>655</v>
+      </c>
+      <c r="C31" t="n">
+        <v>43</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E31" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>256</v>
+      </c>
+      <c r="H31" t="n">
+        <v>128</v>
+      </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K31" t="n">
+        <v>20</v>
+      </c>
+      <c r="L31" t="n">
+        <v>10</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O31" t="b">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.9913</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0.9791</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>655</v>
+      </c>
+      <c r="C32" t="n">
+        <v>43</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>256</v>
+      </c>
+      <c r="H32" t="n">
+        <v>128</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K32" t="n">
+        <v>20</v>
+      </c>
+      <c r="L32" t="n">
+        <v>10</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N32" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.9913</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0.9878</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>655</v>
+      </c>
+      <c r="C33" t="n">
+        <v>43</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>lightglue</t>
+        </is>
+      </c>
+      <c r="E33" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>256</v>
+      </c>
+      <c r="H33" t="n">
+        <v>128</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K33" t="n">
+        <v>20</v>
+      </c>
+      <c r="L33" t="n">
+        <v>10</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O33" t="b">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.9043</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.9565</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0.8963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>